<commit_message>
Added new raw data.
</commit_message>
<xml_diff>
--- a/raw/20260305_r5_SG_Prioscout_NorCWD_RT-QuIC.xlsx
+++ b/raw/20260305_r5_SG_Prioscout_NorCWD_RT-QuIC.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MNPRO\Desktop\RT-QuIC Data\Sarah's RT-QuIC Data\2026\20260305_r5_SG_Prioscout_NorCWD_RT-QuIC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rowde002\Documents\Projects\canadian-reindeer-sentinels\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8EE9D44E-148D-4B8B-9EFF-DFE1DD7D5065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B11F2C16-4D8C-483A-9262-83688A6F1801}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{9DAE0357-5F1A-4A07-A427-8C093CD4A6CC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9DAE0357-5F1A-4A07-A427-8C093CD4A6CC}"/>
   </bookViews>
   <sheets>
     <sheet name="Microplate Cycle 1 (0 h)" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="171">
   <si>
     <t>User: USER</t>
   </si>
@@ -550,6 +550,9 @@
   </si>
   <si>
     <t>3. Dilutions</t>
+  </si>
+  <si>
+    <t>S-2192</t>
   </si>
 </sst>
 </file>
@@ -1672,7 +1675,7 @@
         <v>144</v>
       </c>
       <c r="M27" s="13" t="s">
-        <v>145</v>
+        <v>170</v>
       </c>
       <c r="O27" s="21"/>
     </row>
@@ -1713,8 +1716,8 @@
       <c r="L28" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="M28" s="15" t="s">
-        <v>145</v>
+      <c r="M28" s="13" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -1754,8 +1757,8 @@
       <c r="L29" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="M29" s="15" t="s">
-        <v>145</v>
+      <c r="M29" s="13" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
@@ -1795,8 +1798,8 @@
       <c r="L30" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="M30" s="15" t="s">
-        <v>145</v>
+      <c r="M30" s="13" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">

</xml_diff>